<commit_message>
feat(presupuestos): actualizar P-2026-0045 configuracion en L con base tubular y 3 escalones de arranque
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0045-escalera-metalica-forrada-madera-iroco-costel-pindea/presupuesto.xlsx
+++ b/presupuestos/P-2026-0045-escalera-metalica-forrada-madera-iroco-costel-pindea/presupuesto.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-2026-0045 Escalera Iroco" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-2026-0045 Escalera L Iroco" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,11 +514,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -535,7 +535,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0045</t>
+          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0045 (REV. 1)</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Escalera metálica volada sobre pletina de pared, peldaños de tubo 50x50x5 forrados en Iroko y barandilla de varillas a viga de madera</t>
+          <t>Escalera metálica en L: base tubular arranque (3 escalones), tramo volado pletina mural, forrado Iroko y barandilla varillas a viga de techo</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Zanca pletina 150x12 mm amurada a pared | Ménsulas tubo 50x50x5 mm con tuercas remache M10 | Varillas Ø10 mm a angular en viga de techo | Forrado en madera maciza de Iroko (huella 38 mm)</t>
+          <t>Escalera en L | Base tubular para 3 escalones de arranque | Zanca pletina 150x12 mm amurada a pared | Ménsulas tubo 50x50x5 mm con tuercas remache M10 | Varillas Ø10 mm a angular en viga de madera | Forrado integral de 19 peldaños en madera maciza de Iroko</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Toma de medidas, replanteo láser in situ y desarrollo de planos de despiece milimétricos (verificación de aplomados, cota de viga y cumplimiento CTE DB-SUA)</t>
+          <t>Toma de medidas, replanteo láser in situ y desarrollo de planos de despiece para configuración en L (giro a 90° en arranque, plomos, cota de viga de madera y cumplimiento CTE DB-SUA)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -651,7 +651,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="F12" s="12">
         <f>D12*E12</f>
@@ -666,7 +666,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Fabricación en taller de zanca pletina mural (150x12 mm S275JR) y 16 ménsulas en tubo cuadrado estructural de 50x50x5 mm soldadas, con tuercas remache M10 insertadas</t>
+          <t>Fabricación de base tubular estructural para arranque en L de 3 escalones (chasis soldado en tubo 80x40x3 y 50x50x3 mm S275JR, pletinas de anclaje a solera y encuentro con zanca mural)</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -678,7 +678,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>3850</v>
+        <v>1150</v>
       </c>
       <c r="F13" s="12">
         <f>D13*E13</f>
@@ -693,7 +693,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Barandilla vertical suspendida de varillas calibradas/roscadas Ø10 mm (32 uds para hueco &lt; 10 cm) y perfil angular superior L 60x40x5 mm fijado a viga de madera con tuercas ciegas</t>
+          <t>Fabricación en taller de zanca pletina mural (150x12 mm S275JR) y 16 ménsulas en tubo cuadrado estructural de 50x50x5 mm soldadas, con tuercas remache M10 de alta resistencia insertadas</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -705,7 +705,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>1950</v>
+        <v>3850</v>
       </c>
       <c r="F14" s="12">
         <f>D14*E14</f>
@@ -720,7 +720,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Tratamiento anticorrosivo y lacado de cerrajería en taller: limpieza, imprimación epoxi fosfatante antioxidante y esmalte poliuretano horno (RAL 7016 / 9005 texturado)</t>
+          <t>Barandilla vertical suspendida de varillas calibradas/roscadas Ø10 mm (32 uds para hueco &lt; 10 cm) y perfil angular superior L 60x40x5 mm fijado a viga de madera con tuercas ciegas decorativas</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -732,7 +732,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>880</v>
+        <v>1950</v>
       </c>
       <c r="F15" s="12">
         <f>D15*E15</f>
@@ -747,7 +747,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Forrado integral de 16 peldaños en Madera Maciza de Iroko de 1ª calidad seleccionada (huella 38 mm, frentes 20 mm, cajeado para ocultar tubos y 3 capas de barniz poliuretano alto tránsito)</t>
+          <t>Tratamiento anticorrosivo y lacado de toda la cerrajería en taller: limpieza, imprimación epoxi fosfatante antioxidante y esmalte poliuretano secado al horno (RAL 7016 / 9005 texturado)</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -759,7 +759,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>4250</v>
+        <v>980</v>
       </c>
       <c r="F16" s="12">
         <f>D16*E16</f>
@@ -774,7 +774,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Transporte a obra en Menorca, fijación química estructural a muro maestro con resina viniléster y varillas M14, anclaje superior en viga, tensado de varillas, pegado de peldaños y remates</t>
+          <t>Forrado integral de 19 peldaños en Madera Maciza de Iroko de 1ª calidad seleccionada (3 en base arranque + 16 en tramo volado; huella 38 mm, frentes 20 mm y 3 capas barniz poliuretano tránsito)</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -786,96 +786,123 @@
         <v>1</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>2480</v>
+        <v>4980</v>
       </c>
       <c r="F17" s="12">
         <f>D17*E17</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>Base Imponible:</t>
-        </is>
-      </c>
-      <c r="F19" s="14">
-        <f>SUM(F12:F17)</f>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Transporte a obra en Menorca, fijación química a solera y muro maestro, montaje de angular en viga de madera, tensado de varillas, pegado elastomérico de peldaños de Iroko y remates</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>2780</v>
+      </c>
+      <c r="F18" s="12">
+        <f>D18*E18</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="E20" s="13" t="inlineStr">
         <is>
+          <t>Base Imponible:</t>
+        </is>
+      </c>
+      <c r="F20" s="14">
+        <f>SUM(F12:F18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" s="13" t="inlineStr">
+        <is>
           <t>I.V.A. (21%):</t>
         </is>
       </c>
-      <c r="F20" s="14">
-        <f>F19*0.21</f>
+      <c r="F21" s="14">
+        <f>F20*0.21</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="E21" s="15" t="inlineStr">
+    <row r="22">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>TOTAL PRESUPUESTO:</t>
         </is>
       </c>
-      <c r="F21" s="16">
-        <f>F19+F20</f>
+      <c r="F22" s="16">
+        <f>F20+F21</f>
         <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>CONDICIONES COMERCIALES Y GARANTÍAS</t>
-        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>• Forma de pago:</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>40% a la formalización del pedido y replanteo, 30% a la finalización de estructura y madera en taller, y 30% a la finalización y entrega en obra</t>
+          <t>CONDICIONES COMERCIALES Y GARANTÍAS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>• Garantía:</t>
+          <t>• Forma de pago:</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>2 años en estructura de acero, cerrajería, fijaciones y acabados según normativa vigente</t>
+          <t>40% a la formalización del pedido y replanteo, 30% a la finalización de estructura y madera en taller, y 30% a la finalización y entrega en obra</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>• Plazo de entrega:</t>
+          <t>• Garantía:</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>4 a 5 semanas para taller de cerrajería y ebanistería; montaje en obra de 3 a 4 jornadas laborables</t>
+          <t>2 años en estructura de acero, cerrajería, fijaciones y acabados según normativa vigente</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t>• Plazo de entrega:</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>4 a 5 semanas para taller de cerrajería y ebanistería; montaje en obra de 4 jornadas laborables</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>• Validez:</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>30 días naturales desde la fecha de emisión</t>
         </is>

</xml_diff>

<commit_message>
fix(presupuestos): actualizar P-2026-0045 forma de pago 100% y fijaciones/tuercas a definir
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0045-escalera-metalica-forrada-madera-iroco-costel-pindea/presupuesto.xlsx
+++ b/presupuestos/P-2026-0045-escalera-metalica-forrada-madera-iroco-costel-pindea/presupuesto.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -535,7 +535,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0045 (REV. 1)</t>
+          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0045 (REV. 2)</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Escalera metálica en L: base tubular arranque (3 escalones), tramo volado pletina mural, forrado Iroko y barandilla varillas a viga de techo</t>
+          <t>Escalera en L: base tubular arranque (3 escalones), tramo volado pletina mural, forrado Iroko y varillas a viga de madera (fijaciones a definir)</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Escalera en L | Base tubular para 3 escalones de arranque | Zanca pletina 150x12 mm amurada a pared | Ménsulas tubo 50x50x5 mm con tuercas remache M10 | Varillas Ø10 mm a angular en viga de madera | Forrado integral de 19 peldaños en madera maciza de Iroko</t>
+          <t>Escalera en L | Base tubular para 3 escalones de arranque | Zanca pletina 150x12 mm amurada a pared | Tubos 50x50x5 mm | Varillas Ø10 mm a viga de madera | Forrado 19 peldaños en Iroko macizo | Detalles de tuercas y fijaciones a definir</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Toma de medidas, replanteo láser in situ y desarrollo de planos de despiece para configuración en L (giro a 90° en arranque, plomos, cota de viga de madera y cumplimiento CTE DB-SUA)</t>
+          <t>Toma de medidas, replanteo láser in situ y desarrollo de planos de despiece para configuración en L (giro a 90° en arranque, verificación de plomos, cota de viga y definición de detalles de tuercas y fijaciones)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Fabricación de base tubular estructural para arranque en L de 3 escalones (chasis soldado en tubo 80x40x3 y 50x50x3 mm S275JR, pletinas de anclaje a solera y encuentro con zanca mural)</t>
+          <t>Fabricación de base tubular estructural para arranque en L de 3 escalones (chasis soldado en tubo 80x40x3 y 50x50x3 mm S275JR, pletinas de anclaje a solera y encuentro con zanca mural; fijaciones a definir)</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Fabricación en taller de zanca pletina mural (150x12 mm S275JR) y 16 ménsulas en tubo cuadrado estructural de 50x50x5 mm soldadas, con tuercas remache M10 de alta resistencia insertadas</t>
+          <t>Fabricación en taller de zanca pletina mural (150x12 mm S275JR) y 16 ménsulas en tubo cuadrado estructural de 50x50x5 mm soldadas, con tuercas remache insertadas (tipo y métrica a definir)</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Barandilla vertical suspendida de varillas calibradas/roscadas Ø10 mm (32 uds para hueco &lt; 10 cm) y perfil angular superior L 60x40x5 mm fijado a viga de madera con tuercas ciegas decorativas</t>
+          <t>Barandilla vertical suspendida de varillas calibradas/roscadas Ø10 mm (32 uds para hueco &lt; 10 cm) y perfil angular superior L 60x40x5 mm fijado a viga de madera (detalles de tuercas y fijaciones a definir)</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Transporte a obra en Menorca, fijación química a solera y muro maestro, montaje de angular en viga de madera, tensado de varillas, pegado elastomérico de peldaños de Iroko y remates</t>
+          <t>Transporte a obra en Menorca, fijaciones a solera, muro y viga de madera, montaje de varillas, pegado elastomérico de peldaños de Iroko y remates (sistemas de fijación y tuercas a definir)</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -866,43 +866,55 @@
           <t>• Forma de pago:</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>40% a la formalización del pedido y replanteo, 30% a la finalización de estructura y madera en taller, y 30% a la finalización y entrega en obra</t>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>100% a la aceptación del presupuesto</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>• Garantía:</t>
+          <t>• Fijaciones / tuercas:</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>2 años en estructura de acero, cerrajería, fijaciones y acabados según normativa vigente</t>
+          <t>Detalles constructivos de tuercas y sistemas de fijación a muro, solera y viga a definir en replanteo</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>• Plazo de entrega:</t>
+          <t>• Garantía:</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>4 a 5 semanas para taller de cerrajería y ebanistería; montaje en obra de 4 jornadas laborables</t>
+          <t>2 años en estructura de acero, cerrajería, fijaciones y acabados según normativa vigente</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>• Plazo de entrega:</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>4 a 5 semanas para taller de cerrajería y ebanistería; montaje en obra de 4 jornadas laborables</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
           <t>• Validez:</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>30 días naturales desde la fecha de emisión</t>
         </is>

</xml_diff>

<commit_message>
feat(presupuestos): incorporar 10% comision oculta en partidas para constructor P-2026-0045
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0045-escalera-metalica-forrada-madera-iroco-costel-pindea/presupuesto.xlsx
+++ b/presupuestos/P-2026-0045-escalera-metalica-forrada-madera-iroco-costel-pindea/presupuesto.xlsx
@@ -535,7 +535,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0045 (REV. 2)</t>
+          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0045 (REV. 3)</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>520</v>
+        <v>572</v>
       </c>
       <c r="F12" s="12">
         <f>D12*E12</f>
@@ -678,7 +678,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>1150</v>
+        <v>1265</v>
       </c>
       <c r="F13" s="12">
         <f>D13*E13</f>
@@ -705,7 +705,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>3850</v>
+        <v>4235</v>
       </c>
       <c r="F14" s="12">
         <f>D14*E14</f>
@@ -732,7 +732,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>1950</v>
+        <v>2145</v>
       </c>
       <c r="F15" s="12">
         <f>D15*E15</f>
@@ -759,7 +759,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>980</v>
+        <v>1078</v>
       </c>
       <c r="F16" s="12">
         <f>D16*E16</f>
@@ -786,7 +786,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>4980</v>
+        <v>5478</v>
       </c>
       <c r="F17" s="12">
         <f>D17*E17</f>
@@ -813,7 +813,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>2780</v>
+        <v>3058</v>
       </c>
       <c r="F18" s="12">
         <f>D18*E18</f>

</xml_diff>